<commit_message>
Trim quotation scope per review
- 대관료(실비정산) 제외, 통천 현수막·현장 연출 소품·온라인 모집 삭제(과업내용서 미기재)
- 기획·운영 총괄을 PM + 운영 인력 3인(마마미디어 1인 포함)으로 정리
- 참여단 관리 50명 규모 비례 조정, 접수 인력 '25 단가 적용, 결과보고서 상향

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018WmVGxh2eujqtEGBBBdyNp
</commit_message>
<xml_diff>
--- a/2026_취약노동자원탁회의_결과보고회/[내부]견적_산출근거_2025실적비교.xlsx
+++ b/2026_취약노동자원탁회의_결과보고회/[내부]견적_산출근거_2025실적비교.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -498,49 +498,49 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>프로젝트 총괄(PM) 인건비</t>
+          <t>행사장 대관료</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>40만원 × 5일</t>
+          <t>회당 181.9만원</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>92만원 × 1인 × 2회</t>
+          <t>제외</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) PM(책임연구원) 단가 920,000원/회</t>
+          <t>실비 정산 항목 — 견적에서 제외, 별도 정산</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>지혜의영토</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>운영 인력 인건비</t>
+          <t>프로젝트 총괄(PM) 인건비</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>30만원 × 8일</t>
+          <t>40만원 × 5일</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>71만원 × 2인 × 2회</t>
+          <t>92만원 × 1인 × 2회</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 운영인력 단가 710,000원(전과정 투입). '25년 100인 3인 → 50인 2인</t>
+          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) PM(책임연구원) 920,000원/회</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -552,49 +552,49 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>참여단 관리</t>
+          <t>운영 인력 인건비</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>25만원 × 8일</t>
+          <t>30만원 × 8일 + 마마 현장PM 84.9만원×2</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>120만원 × 2회</t>
+          <t>71만원 × 3인 × 2회 (마마 1인 포함)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 참여단 관리(RSVP·수당지급명세서) 1,200,000원/식</t>
+          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 운영인력 710,000원(전과정 투입). 마마미디어 현장 운영 PM을 운영 인력으로 통합</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>지혜의영토</t>
+          <t>지혜의영토 2 / 마마 1</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>온라인 모집 시스템·홍보</t>
+          <t>참여단 관리</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>15만원 × 2회</t>
+          <t>120만원 × 2회</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>30만원 × 2회</t>
+          <t>40만원 × 2회</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 온라인 모집 시스템 600,000원(100인) → 50인 규모 절반</t>
+          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 1,200,000원(150명) → 50명 규모 비례(1/3). 홍보방안 수립 포함</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -606,22 +606,22 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>접수 소모품</t>
+          <t>등록·접수 안내 인력</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>10만원 × 2회</t>
+          <t>20만원 × 2인 × 2회</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>20만원 × 2회</t>
+          <t>15만원 × 2인 × 2회</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 소모품 200,000원 / '25.11.25 600,000원(150인)</t>
+          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 리셉션·플로어 지원 150,000원/인</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -633,27 +633,27 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>행사보험</t>
+          <t>온라인 모집 시스템·홍보</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>30만원 × 2회</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>삭제</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>과업내용서에 없음(‘홍보 방안 수립’만 있음 → 참여단 관리에 포함)</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
           <t>-</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>15만원 × 2회 (신규)</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 행사보험 300,000원(100인) → 50인 규모</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>지혜의영토</t>
         </is>
       </c>
     </row>
@@ -665,17 +665,17 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>20만원 × 2회</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>20만원 × 2회 (신규)</t>
+          <t>50만원 × 2회</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 행사 결과보고서 200,000원/회</t>
+          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 200,000원 + 분석·결과정리 750,000원 항목 참고, 의견 정리·사진 포함</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -687,88 +687,88 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>출장비(운영 인력)</t>
+          <t>무대 배경 통천 현수막</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>80만원(2회 합산)</t>
+          <t>27.5만원 × 2회</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>부산 60만 + 대전 25만</t>
+          <t>삭제</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>KTX 왕복(부산 약 12만·대전 약 5만/인) × 3인 + 부산 숙박 2실, 현지교통</t>
+          <t>과업내용서에 ‘현수막’만 명시, 통천 없음</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>지혜의영토</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>참석자 다과·생수</t>
+          <t>현장 연출 소품</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>1.2만원/인</t>
+          <t>33만원 × 2회</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>1.65만원/인 (VAT 포함)</t>
+          <t>삭제</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 다과 실지출 613,100원/40인 = 1.53만원/인 ('25.11.25 견적 1.2만원/인)</t>
+          <t>과업내용서에 없음(‘스크린·조명·음향 등 연출’만 명시)</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>마마미디어</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>사전 티타임 준비</t>
+          <t>접수 소모품</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>16.5만원/회</t>
+          <t>10만원 × 2회</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>22만원/회</t>
+          <t>20만원 × 2회</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 내빈 다과(오설록·태극당 등) 실지출 반영</t>
+          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 소모품 200,000원</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>마마미디어</t>
+          <t>지혜의영토</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>무대 배경 통천 현수막</t>
+          <t>행사보험</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -778,66 +778,66 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>27.5만원 × 2회 (신규)</t>
+          <t>15만원 × 2회</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 무대월 통천·가림막 현수막 제작 실적</t>
+          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 행사보험 300,000원(100인) → 50인 규모</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>마마미디어</t>
+          <t>지혜의영토</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>배너</t>
+          <t>출장비(운영 인력)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2개/회</t>
+          <t>80만원(2회 합산)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>4개/회</t>
+          <t>부산 60만 + 대전 25만</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 배너 6개 제작(건물 입구·동선 안내)</t>
+          <t>KTX 왕복(부산 약 12만·대전 약 5만/인) × 3인 + 부산 숙박 2실, 현지교통</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>마마미디어</t>
+          <t>지혜의영토</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>폼보드</t>
+          <t>참석자 다과·생수</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>2개/회</t>
+          <t>1.2만원/인</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>3개/회</t>
+          <t>1.65만원/인 (VAT 포함)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 연단보드 2 + 이젤보드 1</t>
+          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 다과 실지출 613,100원/40인 = 1.53만원/인</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -849,39 +849,120 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>현장 연출 소품</t>
+          <t>사전 티타임 준비</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
+          <t>16.5만원/회</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>22만원/회</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 내빈 다과 실지출 반영</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>마마미디어</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>배너 / 폼보드</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>2개 / 2개 (회당)</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>4개 / 3개 (회당)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 배너 6개, 연단보드 2 + 이젤보드 1 제작</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>마마미디어</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>사진·영상 제작 4종</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>33만원 × 2회 (신규)</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 포토존 25만(견적 10만) + 테이블보 6.3만 + 이젤 3만 정산</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>마마 원견적 단가 × 1.2127</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>마마미디어 견적(사진영상 50만·영상촬영 50만·사진 40만·편집 70만) VAT·관리비·이윤 포함 환산. 참고: '25.10.22 영상·사진 80만(30명), '25.11.25 500만(100인)</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>마마미디어</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>현장 운영 보조</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>마마 원견적 20만원/인 → 24.3만원</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>마마미디어 견적(행사보조·마이크 전달 2인) 환산. 참고: '25 진행보조·리셉션 15만원/인 → 지방 출장 감안 유지</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>마마미디어</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>※ 시사점: '25.10.22 행사는 제작물(견적 150만 → 정산 250만)과 포토존·다과에서 초과가 발생해 90만원을 다음 견적('25.11.25)에 추가 반영함.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">   이번 견적은 해당 항목을 정산 실적 수준으로 사전 반영하여 초과 리스크를 줄임. 인건비는 재단에 기제출·승인된 회당 단가를 그대로 적용.</t>
         </is>

</xml_diff>

<commit_message>
Align quotation with Mama Media revised quote and draft reply email
- 마마미디어 수정견적(10.20, 20,610,000원) 기준 환산단가(올림) 적용
- 명패 50개·배너·폼보드·명찰 단가, 운영 인력 85만원(마마 PM 이상)으로 조정
- 김잔디 위원 회신 메일 초안 추가

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018WmVGxh2eujqtEGBBBdyNp
</commit_message>
<xml_diff>
--- a/2026_취약노동자원탁회의_결과보고회/[내부]견적_산출근거_2025실적비교.xlsx
+++ b/2026_취약노동자원탁회의_결과보고회/[내부]견적_산출근거_2025실적비교.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -557,17 +557,17 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>30만원 × 8일 + 마마 현장PM 84.9만원×2</t>
+          <t>30만원 × 8일 + 마마 현장PM</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>71만원 × 3인 × 2회 (마마 1인 포함)</t>
+          <t>85만원 × 3인 × 2회 (마마 1인 포함)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 운영인력 710,000원(전과정 투입). 마마미디어 현장 운영 PM을 운영 인력으로 통합</t>
+          <t>마마미디어 수정견적 총괄기획·PM 70만원 환산(848,647원) 이상으로 통일. 참고: '25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 운영인력 710,000원</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -579,49 +579,49 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>참여단 관리</t>
+          <t>배너·폼보드·명패·명찰</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>120만원 × 2회</t>
+          <t>6만·4.2만·5,500·2,750원</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>40만원 × 2회</t>
+          <t>9.7만·6.1만·6,100·3,700원</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 1,200,000원(150명) → 50명 규모 비례(1/3). 홍보방안 수립 포함</t>
+          <t>마마미디어 수정견적(10.20) 단가 환산. 명패 회당 15→50개(마마 기준)</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>지혜의영토</t>
+          <t>마마미디어</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>등록·접수 안내 인력</t>
+          <t>참여단 관리</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>20만원 × 2인 × 2회</t>
+          <t>120만원 × 2회</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>15만원 × 2인 × 2회</t>
+          <t>40만원 × 2회</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 리셉션·플로어 지원 150,000원/인</t>
+          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 1,200,000원(150명) → 50명 규모 비례(1/3). 홍보방안 수립 포함</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -633,93 +633,93 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>온라인 모집 시스템·홍보</t>
+          <t>등록·접수 안내 인력</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>30만원 × 2회</t>
+          <t>20만원 × 2인 × 2회</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>삭제</t>
+          <t>15만원 × 2인 × 2회</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>과업내용서에 없음(‘홍보 방안 수립’만 있음 → 참여단 관리에 포함)</t>
+          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 리셉션·플로어 지원 150,000원/인</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>지혜의영토</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>행사 결과보고서</t>
+          <t>온라인 모집 시스템·홍보</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>20만원 × 2회</t>
+          <t>30만원 × 2회</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>50만원 × 2회</t>
+          <t>삭제</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 200,000원 + 분석·결과정리 750,000원 항목 참고, 의견 정리·사진 포함</t>
+          <t>과업내용서에 없음(‘홍보 방안 수립’만 있음 → 참여단 관리에 포함)</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>지혜의영토</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>무대 배경 통천 현수막</t>
+          <t>행사 결과보고서</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>27.5만원 × 2회</t>
+          <t>20만원 × 2회</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>삭제</t>
+          <t>50만원 × 2회</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>과업내용서에 ‘현수막’만 명시, 통천 없음</t>
+          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 200,000원 + 분석·결과정리 750,000원 항목 참고, 의견 정리·사진 포함</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>지혜의영토</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>현장 연출 소품</t>
+          <t>무대 배경 통천 현수막</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>33만원 × 2회</t>
+          <t>27.5만원 × 2회</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>과업내용서에 없음(‘스크린·조명·음향 등 연출’만 명시)</t>
+          <t>과업내용서에 ‘현수막’만 명시, 통천 없음</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -741,49 +741,49 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>접수 소모품</t>
+          <t>현장 연출 소품</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>10만원 × 2회</t>
+          <t>33만원 × 2회</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>20만원 × 2회</t>
+          <t>삭제</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 소모품 200,000원</t>
+          <t>과업내용서에 없음(‘스크린·조명·음향 등 연출’만 명시)</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>지혜의영토</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>행사보험</t>
+          <t>접수 소모품</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10만원 × 2회</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>15만원 × 2회</t>
+          <t>20만원 × 2회</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 행사보험 300,000원(100인) → 50인 규모</t>
+          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 소모품 200,000원</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -795,22 +795,22 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>출장비(운영 인력)</t>
+          <t>행사보험</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>80만원(2회 합산)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>부산 60만 + 대전 25만</t>
+          <t>15만원 × 2회</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>KTX 왕복(부산 약 12만·대전 약 5만/인) × 3인 + 부산 숙박 2실, 현지교통</t>
+          <t>'25.11.25 우리노동부 타운홀미팅 재단 제출 견적(지혜의영토) 행사보험 300,000원(100인) → 50인 규모</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -822,49 +822,49 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>참석자 다과·생수</t>
+          <t>출장비(운영 인력)</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>1.2만원/인</t>
+          <t>80만원(2회 합산)</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>1.65만원/인 (VAT 포함)</t>
+          <t>부산 60만 + 대전 25만</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 다과 실지출 613,100원/40인 = 1.53만원/인</t>
+          <t>KTX 왕복(부산 약 12만·대전 약 5만/인) × 3인 + 부산 숙박 2실, 현지교통</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>마마미디어</t>
+          <t>지혜의영토</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>사전 티타임 준비</t>
+          <t>참석자 다과·생수</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>16.5만원/회</t>
+          <t>1.2만원/인</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>22만원/회</t>
+          <t>1.65만원/인 (VAT 포함)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 내빈 다과 실지출 반영</t>
+          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 다과 실지출 613,100원/40인 = 1.53만원/인</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -876,22 +876,22 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>배너 / 폼보드</t>
+          <t>사전 티타임 준비</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>2개 / 2개 (회당)</t>
+          <t>16.5만원/회</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>4개 / 3개 (회당)</t>
+          <t>22만원/회</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 배너 6개, 연단보드 2 + 이젤보드 1 제작</t>
+          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 내빈 다과 실지출 반영</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -903,22 +903,22 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>사진·영상 제작 4종</t>
+          <t>배너 / 폼보드</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2개 / 2개 (회당)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>마마 원견적 단가 × 1.2127</t>
+          <t>4개 / 3개 (회당)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>마마미디어 견적(사진영상 50만·영상촬영 50만·사진 40만·편집 70만) VAT·관리비·이윤 포함 환산. 참고: '25.10.22 영상·사진 80만(30명), '25.11.25 500만(100인)</t>
+          <t>'25.10.22 콘텐츠·미디어 종사자 간담회 정산(견적 550만→정산 640만, 90만 초과) 배너 6개, 연단보드 2 + 이젤보드 1 제작</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -930,39 +930,66 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>사진·영상 제작 4종</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>마마 원견적 단가 × 1.2127</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>마마미디어 견적(사진영상 50만·영상촬영 50만·사진 40만·편집 70만) VAT·관리비·이윤 포함 환산. 참고: '25.10.22 영상·사진 80만(30명), '25.11.25 500만(100인)</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>마마미디어</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>현장 운영 보조</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>마마 원견적 20만원/인 → 24.3만원</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>마마미디어 견적(행사보조·마이크 전달 2인) 환산. 참고: '25 진행보조·리셉션 15만원/인 → 지방 출장 감안 유지</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>마마미디어</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>※ 시사점: '25.10.22 행사는 제작물(견적 150만 → 정산 250만)과 포토존·다과에서 초과가 발생해 90만원을 다음 견적('25.11.25)에 추가 반영함.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">   이번 견적은 해당 항목을 정산 실적 수준으로 사전 반영하여 초과 리스크를 줄임. 인건비는 재단에 기제출·승인된 회당 단가를 그대로 적용.</t>
         </is>

</xml_diff>